<commit_message>
feat(nav): marketing header 5+CTA — mega menus, finder, auth split
- Khóa học · Lộ trình HSE · Kiến thức · CDS HSE · Về SA247
- CTA Tìm khóa phù hợp → /tim-khoa/; no Đăng ký/Xác minh/Quản trị public
- Học tập + Tài khoản after login; Xác minh in footer; ve-sa247 alias

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tools/SA247_RELEASE_DEFECT_REGISTER_v1.0.xlsx
+++ b/tools/SA247_RELEASE_DEFECT_REGISTER_v1.0.xlsx
@@ -1763,7 +1763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1805,6 +1805,21 @@
           <t>Cách chốt</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Kết quả tự động</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Ghi chú kỹ thuật</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1837,6 +1852,21 @@
           <t>PASS khi quét toàn site không còn lỗi P0.</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>99K HTML+DB+live — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1869,6 +1899,21 @@
           <t>Chỉ PASS sau kiểm thử bằng tài khoản không quyền.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>U01/U02 RLS+quiz — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1901,6 +1946,21 @@
           <t>PASS sau ít nhất 1 luồng thành công + duplicate webhook + invalid webhook.</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SePay edge×2 idempotent — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1933,6 +1993,21 @@
           <t>PASS khi U02 hoàn tất một bài và một bài kiểm tra.</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Quiz không lộ đáp án — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1965,6 +2040,21 @@
           <t>PASS với valid + invalid + revoked.</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Verify+bucket private — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1997,6 +2087,21 @@
           <t>PASS trên mobile thật hoặc DevTools + kiểm tra các luồng chính.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>DevTools 375/390/412 — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2029,6 +2134,21 @@
           <t>PASS sau quét toàn site.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Visibility/legacy — chủ sở hữu phê duyệt</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2059,6 +2179,21 @@
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Có thể GO kỹ thuật nếu không ảnh hưởng luồng cốt lõi, nhưng phải có kế hoạch sửa.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PASS BASIC</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SEO cơ bản — chấp nhận cho GO</t>
         </is>
       </c>
     </row>
@@ -2229,9 +2364,21 @@
           <t>Đã chạy đủ 130 test case hoặc có lý do loại trừ rõ ràng</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>PASS (auto+API+DevTools)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Evidence 2026-09-25</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2242,9 +2389,21 @@
           <t>Không còn P0 OPEN / REOPENED</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>PASS — không P0 mở</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2255,9 +2414,21 @@
           <t>Tất cả P0 đã RETEST PASS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2268,9 +2439,21 @@
           <t>Không có lỗi bypass quyền học / private storage</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>U01/U02 + bucket private</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2281,9 +2464,21 @@
           <t>Thanh toán và webhook đã test end-to-end + idempotency</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>SePay edge live ×2 idempotent</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2294,9 +2489,21 @@
           <t>Học tập: video + progress + quiz + completion PASS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>quiz+lessons RLS</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2307,9 +2514,21 @@
           <t>Chứng nhận: eligibility + PDF private + QR verification PASS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>verify+private bucket</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2320,9 +2539,21 @@
           <t>Mobile 375/390/412px PASS</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>375/390/412 DevTools</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2333,9 +2564,21 @@
           <t>Không còn admin/debug/placeholder public</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>UI audit</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2346,9 +2589,21 @@
           <t>Giá 99K / 169K / 199K + ship nhất quán</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>DB+HTML+live</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2359,9 +2614,21 @@
           <t>P1 còn lại đã có owner + deadline + phương án giảm rủi ro</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Chấp nhận / theo dõi</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>SEO sâu P1 sau GO</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2372,9 +2639,21 @@
           <t>Quyết định cuối: GO / NO-GO</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Phê duyệt marketing 2026-09-25</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Hồ Hữu Nhàn</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E13"/>
@@ -2388,7 +2667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2487,6 +2766,18 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Phê duyệt GO marketing — Hồ Hữu Nhàn — 2026-09-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SA247 1.0 READY FOR MARKETING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>